<commit_message>
Updates to Sales Report
</commit_message>
<xml_diff>
--- a/DataSources/BudgetPivot.xlsx
+++ b/DataSources/BudgetPivot.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\virve\Documents\Sales Report\Data Sources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opilane\Documents\andmetarkus2026\DataSources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAE10B5-45A0-45B6-9425-907757C8EB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765AE73F-E846-4FA5-8D1D-604425AF8151}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A448E068-D00D-4D43-BCF5-A1C382574009}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{A448E068-D00D-4D43-BCF5-A1C382574009}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -54,7 +54,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -450,13 +450,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E93814E-81F9-4C2C-94BB-2C1E76FE9B86}">
   <dimension ref="A1:BU4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="73" width="9.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:73" ht="15">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -677,7 +677,7 @@
         <v>45992</v>
       </c>
     </row>
-    <row r="2" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:73">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -898,7 +898,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="3" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:73">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="4" spans="1:73" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:73">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1346,15 +1346,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D8BC7FD0AA6EEA499D9B093AC6E3EACC" ma:contentTypeVersion="9" ma:contentTypeDescription="Loo uus dokument" ma:contentTypeScope="" ma:versionID="411f39168d3a60f88cab6123ec507e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="761d0801-ebf0-405d-ba89-5fd93677c3c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a27d5aba181a0c08311b137ab24f3109" ns3:_="">
     <xsd:import namespace="761d0801-ebf0-405d-ba89-5fd93677c3c3"/>
@@ -1528,6 +1519,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1537,14 +1537,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FBE3A50-6F1A-440E-B3F5-0B26957AC0AF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F257E011-7AA5-473B-9963-C74D274B0489}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1558,6 +1550,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FBE3A50-6F1A-440E-B3F5-0B26957AC0AF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>